<commit_message>
fix: UISprite 表 Id 对齐 Item.IconPath（icon_sword/icon_potion）
Item.IconPath 的值是 icon_sword / icon_potion，UISprite.Id 原来写成 item_icon_sword
对不上。统一成 icon_sword 风格，业务直接 GetSpriteById(item.IconPath) 取图。
</commit_message>
<xml_diff>
--- a/Assets/Config/Excel/UISprite.xlsx
+++ b/Assets/Config/Excel/UISprite.xlsx
@@ -420,11 +420,11 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,7 +516,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>逻辑图ID(代码用这个取图)</t>
+          <t>逻辑图ID(代码用这个取图；Item.IconPath 填这里)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,7 +539,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>item_icon_sword</t>
+          <t>icon_sword</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>铁剑图标(演示)</t>
+          <t>铁剑图标(演示，对齐 Item.IconPath)</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>item_icon_potion</t>
+          <t>icon_potion</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>红药水图标(演示)</t>
+          <t>红药水图标(演示，对齐 Item.IconPath)</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>金币(演示)</t>
+          <t>金币按钮(演示)</t>
         </is>
       </c>
     </row>

</xml_diff>